<commit_message>
Refactor project structure: separate backend and frontend
</commit_message>
<xml_diff>
--- a/测试案例.xlsx
+++ b/测试案例.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="10480"/>
+    <workbookView windowWidth="15360" windowHeight="15300"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="45">
   <si>
     <t>模块</t>
   </si>
@@ -58,6 +58,9 @@
     <t>在课表选课提交，对应课程未变色</t>
   </si>
   <si>
+    <t>Deng</t>
+  </si>
+  <si>
     <t>未显示课表</t>
   </si>
   <si>
@@ -79,12 +82,6 @@
     <t>未收到通知</t>
   </si>
   <si>
-    <t>登录权限</t>
-  </si>
-  <si>
-    <t>登陆界面选角色可去掉，不影响登录</t>
-  </si>
-  <si>
     <t>审批</t>
   </si>
   <si>
@@ -146,6 +143,27 @@
   </si>
   <si>
     <t>导出相关班级excel表</t>
+  </si>
+  <si>
+    <t>前端无数据</t>
+  </si>
+  <si>
+    <t>无法选择个人对象</t>
+  </si>
+  <si>
+    <t>无草稿纪录列表</t>
+  </si>
+  <si>
+    <t>上传附件出错</t>
+  </si>
+  <si>
+    <t>同一条请假生成两条记录</t>
+  </si>
+  <si>
+    <t>发起考勤前端功能没有实现</t>
+  </si>
+  <si>
+    <t>考勤签到前后端需要联调</t>
   </si>
 </sst>
 </file>
@@ -1090,12 +1108,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="5"/>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <cols>
-    <col min="2" max="2" width="9.54545454545454"/>
-    <col min="3" max="3" width="14.3909090909091" customWidth="1"/>
-    <col min="4" max="4" width="34.0818181818182" customWidth="1"/>
+    <col min="2" max="2" width="9.5462962962963"/>
+    <col min="3" max="3" width="14.3888888888889" customWidth="1"/>
+    <col min="4" max="4" width="34.0833333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -1131,6 +1149,9 @@
       <c r="D2" t="s">
         <v>8</v>
       </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
@@ -1143,55 +1164,50 @@
         <v>2501301001</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
         <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" t="s">
         <v>20</v>
       </c>
-      <c r="D6" t="s">
-        <v>21</v>
+      <c r="F6" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1205,33 +1221,33 @@
         <v>2501301001</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
         <v>18</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1245,33 +1261,33 @@
         <v>2501301001</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1285,13 +1301,13 @@
         <v>2501301001</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1305,33 +1321,33 @@
         <v>2501301001</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1345,157 +1361,291 @@
         <v>2501301001</v>
       </c>
       <c r="D14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" t="s">
         <v>30</v>
       </c>
-      <c r="B15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" t="s">
-        <v>31</v>
-      </c>
       <c r="E15" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E16" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F16" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="D17" t="s">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D18" t="s">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" t="s">
         <v>34</v>
       </c>
-      <c r="D19" t="s">
-        <v>35</v>
+      <c r="F19" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B20" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E20" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F20" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B21" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E21" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F21" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" t="s">
+        <v>38</v>
+      </c>
+      <c r="E23" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" t="s">
+        <v>40</v>
+      </c>
+      <c r="E25" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" t="s">
+        <v>41</v>
+      </c>
+      <c r="E26" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" t="s">
         <v>14</v>
       </c>
-      <c r="D22" t="s">
-        <v>38</v>
+      <c r="D28" t="s">
+        <v>43</v>
+      </c>
+      <c r="E28" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" t="s">
+        <v>44</v>
+      </c>
+      <c r="E29" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B18 B19 B20 B21 B22 B2:B17 B23:B1048576">
-      <formula1>"学生,辅导员,任课老师,管理员"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A19">
       <formula1>"请假,审批,拉取考勤表,通知任课,登录权限,公假,部署"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A22 A2:A18 A20:A21 A23:A1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A18 A20:A1048576">
       <formula1>"请假,审批,拉取考勤表,通知任课,登录权限,公假"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E22 E2:E21 E23:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576">
+      <formula1>"学生,辅导员,任课老师,管理员"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576">
       <formula1>"是,否"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1509,7 +1659,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -1521,7 +1671,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>